<commit_message>
Add Telegram feed, 2026 program, speakers, videos and novelty review
</commit_message>
<xml_diff>
--- a/data/site/exhibitors.xlsx
+++ b/data/site/exhibitors.xlsx
@@ -6697,10 +6697,18 @@
           <t>+7 (800) 550-37-87</t>
         </is>
       </c>
-      <c r="G99" s="2" t="inlineStr"/>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/vseinstrumentirudiy</t>
+        </is>
+      </c>
       <c r="H99" s="2" t="inlineStr"/>
       <c r="I99" s="2" t="inlineStr"/>
-      <c r="J99" s="2" t="inlineStr"/>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/vseinstrumentirudiy</t>
+        </is>
+      </c>
       <c r="K99" s="2" t="inlineStr">
         <is>
           <t>https://catalog.mitexpo.ru/companies/company/135005-vseinstrumenty-ru-ooo.html</t>
@@ -7039,10 +7047,18 @@
       <c r="D105" s="2" t="inlineStr"/>
       <c r="E105" s="2" t="inlineStr"/>
       <c r="F105" s="2" t="inlineStr"/>
-      <c r="G105" s="2" t="inlineStr"/>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/dvizhok_journal</t>
+        </is>
+      </c>
       <c r="H105" s="2" t="inlineStr"/>
       <c r="I105" s="2" t="inlineStr"/>
-      <c r="J105" s="2" t="inlineStr"/>
+      <c r="J105" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/dvizhok_journal</t>
+        </is>
+      </c>
       <c r="K105" s="2" t="inlineStr">
         <is>
           <t>https://catalog.mitexpo.ru/companies/company/171339-dvizhok.html</t>
@@ -12637,10 +12653,18 @@
       <c r="D195" s="2" t="inlineStr"/>
       <c r="E195" s="2" t="inlineStr"/>
       <c r="F195" s="2" t="inlineStr"/>
-      <c r="G195" s="2" t="inlineStr"/>
+      <c r="G195" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/stroygazeta</t>
+        </is>
+      </c>
       <c r="H195" s="2" t="inlineStr"/>
       <c r="I195" s="2" t="inlineStr"/>
-      <c r="J195" s="2" t="inlineStr"/>
+      <c r="J195" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/stroygazeta</t>
+        </is>
+      </c>
       <c r="K195" s="2" t="inlineStr">
         <is>
           <t>https://catalog.mitexpo.ru/companies/company/171345-stroitelnaya-gazeta.html</t>
@@ -14259,10 +14283,18 @@
           <t>+74842926386</t>
         </is>
       </c>
-      <c r="G221" s="2" t="inlineStr"/>
+      <c r="G221" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/kvt_su</t>
+        </is>
+      </c>
       <c r="H221" s="2" t="inlineStr"/>
       <c r="I221" s="2" t="inlineStr"/>
-      <c r="J221" s="2" t="inlineStr"/>
+      <c r="J221" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/kvt_su</t>
+        </is>
+      </c>
       <c r="K221" s="2" t="inlineStr">
         <is>
           <t>https://catalog.mitexpo.ru/companies/company/84498-kvt-ooo.html</t>

</xml_diff>